<commit_message>
ajuste na meta televendas
</commit_message>
<xml_diff>
--- a/data/meta_faturamento_televendas.xlsx
+++ b/data/meta_faturamento_televendas.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\convenção\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8D1C6B-F67B-47FD-9EEE-4D4D0D92ADD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696B8BD5-A19A-49D3-B601-9DFE61976926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$C$117</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -1662,7 +1665,7 @@
         <v>2476</v>
       </c>
       <c r="C112" s="8">
-        <v>232</v>
+        <v>232000</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1673,7 +1676,7 @@
         <v>2494</v>
       </c>
       <c r="C113" s="8">
-        <v>151</v>
+        <v>151000</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1684,7 +1687,7 @@
         <v>2661</v>
       </c>
       <c r="C114" s="8">
-        <v>198</v>
+        <v>198000</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1695,7 +1698,7 @@
         <v>3465</v>
       </c>
       <c r="C115" s="8">
-        <v>90</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1706,7 +1709,7 @@
         <v>1133</v>
       </c>
       <c r="C116" s="8">
-        <v>90</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1717,7 +1720,7 @@
         <v>3467</v>
       </c>
       <c r="C117" s="8">
-        <v>90</v>
+        <v>90000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajuste de meta televendas
</commit_message>
<xml_diff>
--- a/data/meta_faturamento_televendas.xlsx
+++ b/data/meta_faturamento_televendas.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\convenção\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8D1C6B-F67B-47FD-9EEE-4D4D0D92ADD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696B8BD5-A19A-49D3-B601-9DFE61976926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$C$117</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -1662,7 +1665,7 @@
         <v>2476</v>
       </c>
       <c r="C112" s="8">
-        <v>232</v>
+        <v>232000</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1673,7 +1676,7 @@
         <v>2494</v>
       </c>
       <c r="C113" s="8">
-        <v>151</v>
+        <v>151000</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1684,7 +1687,7 @@
         <v>2661</v>
       </c>
       <c r="C114" s="8">
-        <v>198</v>
+        <v>198000</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1695,7 +1698,7 @@
         <v>3465</v>
       </c>
       <c r="C115" s="8">
-        <v>90</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1706,7 +1709,7 @@
         <v>1133</v>
       </c>
       <c r="C116" s="8">
-        <v>90</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1717,7 +1720,7 @@
         <v>3467</v>
       </c>
       <c r="C117" s="8">
-        <v>90</v>
+        <v>90000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>